<commit_message>
Update BOM and clarify THD units in validation dataset
- hardware/BOM.xlsx: version of 2026-10-15 (total EUR 438.30), with the four
  MakerBeam kit links corrected.
- data/: the THD column holds a fraction (0.11 = 11 %), not a percentage;
  header renamed to "THD (fraction)" and documented in data/README.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/BOM.xlsx
+++ b/hardware/BOM.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Teo\SynologyDrive\Obsidian_COSMIC\04_Rédaction\1_Articles\generator_hardwareX\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Teo\Documents\SynologyDrive\Obsidian_COSMIC\01_Développement\1_Générateur\HVGene_OpenHardware_repo\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC086973-0E3F-4507-BEFE-E8926AAE0053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94657B12-DEE8-4F1F-96D2-BF909A7EBB84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">BOM!$A$1:$K$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">BOM!$A$1:$K$87</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="301">
   <si>
     <t>Category</t>
   </si>
@@ -335,10 +335,10 @@
     <t>Electrical</t>
   </si>
   <si>
-    <t>Alternator</t>
-  </si>
-  <si>
-    <t>custom PCB (JLCPCB manufactured)</t>
+    <t>Custom PCB</t>
+  </si>
+  <si>
+    <t>HVGene inverter/control PCB, bare board (JLCPCB order, KiCAD Gerbers)</t>
   </si>
   <si>
     <t>JLCPCB</t>
@@ -365,13 +365,16 @@
     <t>Voltage Regulator</t>
   </si>
   <si>
-    <t>LM2596 buck converter module (dual board w/ LCD driver)</t>
+    <t>Adjustable CNC buck power-supply module (EC-Buying), 50 V / 20 A max (vendor ratings), controller IC marked CDFM10, with separate LCD control board</t>
   </si>
   <si>
     <t>EC-buying - Amazon</t>
   </si>
   <si>
-    <t>https://www.amazon.com/dp/B0B38GYF74?ref_=ppx_printOD_title_dt_b_fed_asin_title_0_0</t>
+    <t>https://www.amazon.com/dp/B0B38GYF74</t>
+  </si>
+  <si>
+    <t>Controller IC carries only a vendor marking (CDFM10), no published datasheet; ratings as stated by vendor</t>
   </si>
   <si>
     <t>LCD_BUCK_MODULE</t>
@@ -591,6 +594,75 @@
   </si>
   <si>
     <t>https://befr.rs-online.com/web/p/pluggable-terminal-blocks/7900705</t>
+  </si>
+  <si>
+    <t>WIRE_MAINS</t>
+  </si>
+  <si>
+    <t>3G0.75 mm²</t>
+  </si>
+  <si>
+    <t>RND H05VV-F 3-core mains cable, 0.75 mm², 300/500 V, 1.5 m (RND 465-00948)</t>
+  </si>
+  <si>
+    <t>https://befr.rs-online.com/web/p/mains-power-cable/2833214</t>
+  </si>
+  <si>
+    <t>CON_POWER to TXH_240-124 (~0.3 m used, cores separated). Sold as 1.5 m length; if unavailable, AXINDUS H05VV-F 3G0.75 (RS 642-629), 61.24 EUR / 50 m reel</t>
+  </si>
+  <si>
+    <t>WIRE_1.5_RED</t>
+  </si>
+  <si>
+    <t>1.5 mm²</t>
+  </si>
+  <si>
+    <t>RS PRO H07V-K hook-up wire, 1.5 mm², red, 750 V (RS 361-822)</t>
+  </si>
+  <si>
+    <t>https://befr.rs-online.com/web/p/hook-up-wire/0361822</t>
+  </si>
+  <si>
+    <t>Qty in metres; 24 V, V_buck and primary links. Priced pro rata: sold by 100 m reel, 92.86 EUR</t>
+  </si>
+  <si>
+    <t>WIRE_1.5_BLK</t>
+  </si>
+  <si>
+    <t>RS PRO H07V-K hook-up wire, 1.5 mm², black, 750 V (RS 361-787)</t>
+  </si>
+  <si>
+    <t>https://befr.rs-online.com/web/p/hook-up-wire/0361787</t>
+  </si>
+  <si>
+    <t>Qty in metres; 0 V returns and primary links. Priced pro rata: sold by 100 m reel, 92.86 EUR</t>
+  </si>
+  <si>
+    <t>WIRE_1.5_GNYE</t>
+  </si>
+  <si>
+    <t>RS PRO H07V-K hook-up wire, 1.5 mm², green/yellow, 750 V (RS 361-816)</t>
+  </si>
+  <si>
+    <t>https://befr.rs-online.com/web/p/hook-up-wire/0361816</t>
+  </si>
+  <si>
+    <t>Qty in metres; five grounding links to WAGO_5W (~0.85 m). Priced pro rata: sold by 100 m reel, 92.86 EUR</t>
+  </si>
+  <si>
+    <t>WIRE_I2C</t>
+  </si>
+  <si>
+    <t>0.22 mm²</t>
+  </si>
+  <si>
+    <t>RS PRO hook-up wire, 0.22 mm² (24 AWG), 7/0.2 mm, grey PVC (RS 208-1123)</t>
+  </si>
+  <si>
+    <t>https://befr.rs-online.com/web/p/hook-up-wire/2081123</t>
+  </si>
+  <si>
+    <t>Qty in metres; LCD_SCREEN I2C cable (4 x ~12 cm). Priced pro rata: sold by 30.5 m reel, 8.99 EUR</t>
   </si>
   <si>
     <t>Mechanical</t>
@@ -876,7 +948,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -900,6 +972,14 @@
       <sz val="11"/>
       <color rgb="FF0563C1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -964,10 +1044,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -998,8 +1079,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1300,8 +1383,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K83"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K88"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -1314,7 +1397,7 @@
     <col min="10" max="11" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1349,7 +1432,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -1380,7 +1463,7 @@
       </c>
       <c r="K2" s="3"/>
     </row>
-    <row r="3" spans="1:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -1411,7 +1494,7 @@
       </c>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -1442,7 +1525,7 @@
       </c>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -1473,7 +1556,7 @@
       </c>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
@@ -1504,7 +1587,7 @@
       </c>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
@@ -1535,7 +1618,7 @@
       </c>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
@@ -1568,7 +1651,7 @@
       </c>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
@@ -1601,7 +1684,7 @@
       </c>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>11</v>
       </c>
@@ -1634,7 +1717,7 @@
       </c>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
@@ -1667,7 +1750,7 @@
       </c>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -1700,7 +1783,7 @@
       </c>
       <c r="K12" s="3"/>
     </row>
-    <row r="13" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -1733,7 +1816,7 @@
       </c>
       <c r="K13" s="3"/>
     </row>
-    <row r="14" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>11</v>
       </c>
@@ -1766,7 +1849,7 @@
       </c>
       <c r="K14" s="3"/>
     </row>
-    <row r="15" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
@@ -1799,7 +1882,7 @@
       </c>
       <c r="K15" s="3"/>
     </row>
-    <row r="16" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
@@ -1832,7 +1915,7 @@
       </c>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
@@ -1863,7 +1946,7 @@
       </c>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>11</v>
       </c>
@@ -1894,7 +1977,7 @@
       </c>
       <c r="K18" s="3"/>
     </row>
-    <row r="19" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>11</v>
       </c>
@@ -1925,7 +2008,7 @@
       </c>
       <c r="K19" s="3"/>
     </row>
-    <row r="20" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>11</v>
       </c>
@@ -1956,7 +2039,7 @@
       </c>
       <c r="K20" s="3"/>
     </row>
-    <row r="21" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>11</v>
       </c>
@@ -1987,7 +2070,7 @@
       </c>
       <c r="K21" s="3"/>
     </row>
-    <row r="22" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>11</v>
       </c>
@@ -2018,7 +2101,7 @@
       </c>
       <c r="K22" s="3"/>
     </row>
-    <row r="23" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>11</v>
       </c>
@@ -2049,7 +2132,7 @@
       </c>
       <c r="K23" s="3"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>98</v>
       </c>
@@ -2080,7 +2163,7 @@
       </c>
       <c r="K24" s="3"/>
     </row>
-    <row r="25" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>98</v>
       </c>
@@ -2111,7 +2194,7 @@
       </c>
       <c r="K25" s="3"/>
     </row>
-    <row r="26" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>98</v>
       </c>
@@ -2140,14 +2223,16 @@
       <c r="J26" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="K26" s="3"/>
-    </row>
-    <row r="27" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K26" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>104</v>
@@ -2160,22 +2245,22 @@
       <c r="I27" s="2"/>
       <c r="J27" s="3"/>
       <c r="K27" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F28" s="2">
         <v>2</v>
@@ -2190,23 +2275,23 @@
         <v>20</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K28" s="3"/>
     </row>
-    <row r="29" spans="1:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F29" s="2">
         <v>1</v>
@@ -2221,23 +2306,23 @@
         <v>20</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K29" s="3"/>
     </row>
-    <row r="30" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F30" s="2">
         <v>1</v>
@@ -2249,26 +2334,26 @@
         <v>24.99</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K30" s="3"/>
     </row>
-    <row r="31" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F31" s="2">
         <v>1</v>
@@ -2283,19 +2368,19 @@
         <v>20</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K31" s="3"/>
     </row>
-    <row r="32" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="3"/>
@@ -2305,22 +2390,22 @@
       <c r="I32" s="2"/>
       <c r="J32" s="3"/>
       <c r="K32" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F33" s="2">
         <v>1</v>
@@ -2335,23 +2420,23 @@
         <v>15</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="K33" s="3"/>
     </row>
-    <row r="34" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F34" s="2">
         <v>1</v>
@@ -2366,25 +2451,25 @@
         <v>15</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F35" s="2">
         <v>2</v>
@@ -2399,25 +2484,25 @@
         <v>15</v>
       </c>
       <c r="J35" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F36" s="2">
         <v>1</v>
@@ -2432,23 +2517,23 @@
         <v>15</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K36" s="3"/>
     </row>
-    <row r="37" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F37" s="2">
         <v>1</v>
@@ -2463,16 +2548,16 @@
         <v>15</v>
       </c>
       <c r="J37" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K37" s="3"/>
     </row>
-    <row r="38" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>80</v>
@@ -2498,19 +2583,19 @@
       </c>
       <c r="K38" s="3"/>
     </row>
-    <row r="39" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F39" s="2">
         <v>2</v>
@@ -2525,23 +2610,23 @@
         <v>15</v>
       </c>
       <c r="J39" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K39" s="3"/>
     </row>
-    <row r="40" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F40" s="2">
         <v>1</v>
@@ -2556,23 +2641,23 @@
         <v>15</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K40" s="3"/>
     </row>
-    <row r="41" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F41" s="2">
         <v>2</v>
@@ -2587,25 +2672,25 @@
         <v>15</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K41" s="3"/>
     </row>
-    <row r="42" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
         <v>98</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>80</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F42" s="8">
         <v>1</v>
@@ -2620,23 +2705,23 @@
         <v>15</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K42" s="9"/>
     </row>
-    <row r="43" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F43" s="2">
         <v>16</v>
@@ -2651,23 +2736,23 @@
         <v>15</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K43" s="3"/>
     </row>
-    <row r="44" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F44" s="2">
         <v>3</v>
@@ -2682,23 +2767,23 @@
         <v>15</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K44" s="3"/>
     </row>
-    <row r="45" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F45" s="2">
         <v>3</v>
@@ -2713,23 +2798,23 @@
         <v>15</v>
       </c>
       <c r="J45" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K45" s="3"/>
     </row>
-    <row r="46" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D46" s="2"/>
       <c r="E46" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F46" s="2">
         <v>1</v>
@@ -2744,23 +2829,23 @@
         <v>15</v>
       </c>
       <c r="J46" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K46" s="3"/>
     </row>
-    <row r="47" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D47" s="2"/>
       <c r="E47" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F47" s="2">
         <v>2</v>
@@ -2775,23 +2860,23 @@
         <v>15</v>
       </c>
       <c r="J47" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K47" s="3"/>
     </row>
-    <row r="48" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F48" s="2">
         <v>1</v>
@@ -2806,844 +2891,914 @@
         <v>15</v>
       </c>
       <c r="J48" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K48" s="3"/>
     </row>
-    <row r="49" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>185</v>
+        <v>98</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>186</v>
       </c>
       <c r="C49" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="D49" s="2"/>
       <c r="E49" s="3" t="s">
         <v>188</v>
       </c>
       <c r="F49" s="2">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G49" s="4">
-        <v>1.58</v>
+        <v>3.69</v>
       </c>
       <c r="H49" s="4">
-        <v>25.31</v>
+        <v>3.69</v>
       </c>
       <c r="I49" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J49" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="J49" s="5" t="s">
+      <c r="K49" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="K49" s="3"/>
-    </row>
-    <row r="50" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="50" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>185</v>
+        <v>98</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>191</v>
       </c>
       <c r="C50" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="D50" s="2"/>
-      <c r="E50" s="3"/>
+      <c r="E50" s="3" t="s">
+        <v>193</v>
+      </c>
       <c r="F50" s="2">
-        <v>52</v>
-      </c>
-      <c r="G50" s="2"/>
-      <c r="H50" s="2"/>
-      <c r="I50" s="2"/>
-      <c r="J50" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="G50" s="4">
+        <v>0.92859999999999998</v>
+      </c>
+      <c r="H50" s="4">
+        <v>0.93</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J50" s="5" t="s">
+        <v>194</v>
+      </c>
       <c r="K50" s="3" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>185</v>
+        <v>98</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D51" s="2"/>
+        <v>133</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>192</v>
+      </c>
       <c r="E51" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F51" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G51" s="4">
-        <v>5</v>
+        <v>0.92859999999999998</v>
       </c>
       <c r="H51" s="4">
-        <v>20</v>
+        <v>0.93</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>189</v>
+        <v>15</v>
       </c>
       <c r="J51" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="K51" s="3"/>
-    </row>
-    <row r="52" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>198</v>
+      </c>
+      <c r="K51" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>185</v>
+        <v>98</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D52" s="2"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
-      <c r="I52" s="2"/>
-      <c r="J52" s="3"/>
+        <v>133</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F52" s="2">
+        <v>1</v>
+      </c>
+      <c r="G52" s="4">
+        <v>0.92859999999999998</v>
+      </c>
+      <c r="H52" s="4">
+        <v>0.93</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J52" s="5" t="s">
+        <v>202</v>
+      </c>
       <c r="K52" s="3" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>185</v>
+        <v>98</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D53" s="2"/>
-      <c r="E53" s="3"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
-      <c r="I53" s="2"/>
-      <c r="J53" s="3"/>
+        <v>133</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="F53" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G53" s="4">
+        <v>0.29480000000000001</v>
+      </c>
+      <c r="H53" s="4">
+        <v>0.15</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J53" s="5" t="s">
+        <v>207</v>
+      </c>
       <c r="K53" s="3" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="3" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="F54" s="2">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="G54" s="4">
-        <v>0.59</v>
+        <v>1.58</v>
       </c>
       <c r="H54" s="4">
-        <v>2.38</v>
+        <v>25.31</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>189</v>
+        <v>213</v>
       </c>
       <c r="J54" s="5" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="K54" s="3"/>
     </row>
-    <row r="55" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="D55" s="2"/>
-      <c r="E55" s="3" t="s">
-        <v>206</v>
-      </c>
+      <c r="E55" s="3"/>
       <c r="F55" s="2">
-        <v>4</v>
-      </c>
-      <c r="G55" s="4">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="H55" s="4">
-        <v>4.5</v>
-      </c>
-      <c r="I55" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="J55" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="K55" s="3"/>
-    </row>
-    <row r="56" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+      <c r="I55" s="2"/>
+      <c r="J55" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="K55" s="3" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="D56" s="2"/>
       <c r="E56" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="F56" s="2">
+        <v>4</v>
+      </c>
+      <c r="G56" s="4">
+        <v>5</v>
+      </c>
+      <c r="H56" s="4">
+        <v>20</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="J56" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="K56" s="3"/>
+    </row>
+    <row r="57" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="F56" s="2">
-        <v>8</v>
-      </c>
-      <c r="G56" s="4">
-        <v>1.69</v>
-      </c>
-      <c r="H56" s="4">
-        <v>13.53</v>
-      </c>
-      <c r="I56" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="J56" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="K56" s="3"/>
-    </row>
-    <row r="57" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="2" t="s">
-        <v>185</v>
-      </c>
       <c r="B57" s="2" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="D57" s="2"/>
-      <c r="E57" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F57" s="2">
-        <v>8</v>
-      </c>
-      <c r="G57" s="4">
-        <v>1.99</v>
-      </c>
-      <c r="H57" s="4">
-        <v>15.9</v>
-      </c>
-      <c r="I57" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="J57" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="K57" s="3"/>
-    </row>
-    <row r="58" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E57" s="3"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+      <c r="J57" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="K57" s="3" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="D58" s="2"/>
-      <c r="E58" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="F58" s="2">
-        <v>8</v>
-      </c>
-      <c r="G58" s="4">
-        <v>0.64</v>
-      </c>
-      <c r="H58" s="4">
-        <v>5.1100000000000003</v>
-      </c>
-      <c r="I58" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="J58" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="K58" s="3"/>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E58" s="3"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
+      <c r="I58" s="2"/>
+      <c r="J58" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="K58" s="3" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="3" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="F59" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G59" s="4">
-        <v>0.24</v>
+        <v>0.59</v>
       </c>
       <c r="H59" s="4">
-        <v>0.48</v>
+        <v>2.38</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>15</v>
+        <v>213</v>
       </c>
       <c r="J59" s="5" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="K59" s="3"/>
     </row>
-    <row r="60" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="3" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="F60" s="2">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G60" s="4">
-        <v>0.03</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="H60" s="4">
-        <v>0.31</v>
+        <v>4.5</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>189</v>
+        <v>213</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="K60" s="3"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="D61" s="2"/>
       <c r="E61" s="3" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="F61" s="2">
         <v>8</v>
       </c>
       <c r="G61" s="4">
-        <v>0.05</v>
+        <v>1.69</v>
       </c>
       <c r="H61" s="4">
-        <v>0.42</v>
+        <v>13.53</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>15</v>
+        <v>213</v>
       </c>
       <c r="J61" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="K61" s="3"/>
+    </row>
+    <row r="62" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C62" s="2" t="s">
         <v>226</v>
-      </c>
-      <c r="K61" s="3"/>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A62" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>215</v>
       </c>
       <c r="D62" s="2"/>
       <c r="E62" s="3" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="F62" s="2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G62" s="4">
-        <v>0.03</v>
+        <v>1.99</v>
       </c>
       <c r="H62" s="4">
-        <v>0.06</v>
+        <v>15.9</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>15</v>
+        <v>213</v>
       </c>
       <c r="J62" s="5" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="K62" s="3"/>
     </row>
-    <row r="63" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>192</v>
+        <v>239</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="3" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="F63" s="2">
+        <v>8</v>
+      </c>
+      <c r="G63" s="4">
+        <v>0.64</v>
+      </c>
+      <c r="H63" s="4">
+        <v>5.1100000000000003</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="J63" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="K63" s="3"/>
+    </row>
+    <row r="64" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D64" s="2"/>
+      <c r="E64" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="F64" s="2">
         <v>2</v>
       </c>
-      <c r="G63" s="4">
-        <v>0.2</v>
-      </c>
-      <c r="H63" s="4">
-        <v>0.4</v>
-      </c>
-      <c r="I63" s="2" t="s">
+      <c r="G64" s="4">
+        <v>0.24</v>
+      </c>
+      <c r="H64" s="4">
+        <v>0.48</v>
+      </c>
+      <c r="I64" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="J63" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="K63" s="3"/>
-    </row>
-    <row r="64" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D64" s="2"/>
-      <c r="E64" s="3"/>
-      <c r="F64" s="2"/>
-      <c r="G64" s="2"/>
-      <c r="H64" s="2"/>
-      <c r="I64" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="J64" s="3"/>
-      <c r="K64" s="3" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J64" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="K64" s="3"/>
+    </row>
+    <row r="65" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>192</v>
+        <v>239</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="3" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="F65" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G65" s="4">
-        <v>0.56999999999999995</v>
+        <v>0.03</v>
       </c>
       <c r="H65" s="4">
-        <v>1.1399999999999999</v>
+        <v>0.31</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>15</v>
+        <v>213</v>
       </c>
       <c r="J65" s="5" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="K65" s="3"/>
     </row>
-    <row r="66" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>192</v>
+        <v>239</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="3" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="F66" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G66" s="4">
-        <v>1.1100000000000001</v>
+        <v>0.05</v>
       </c>
       <c r="H66" s="4">
-        <v>4.43</v>
+        <v>0.42</v>
       </c>
       <c r="I66" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J66" s="5" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="K66" s="3"/>
     </row>
-    <row r="67" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>192</v>
+        <v>239</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="3" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="F67" s="2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G67" s="4">
-        <v>0.13</v>
+        <v>0.03</v>
       </c>
       <c r="H67" s="4">
-        <v>1.03</v>
+        <v>0.06</v>
       </c>
       <c r="I67" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J67" s="5" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="K67" s="3"/>
     </row>
-    <row r="68" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>192</v>
+        <v>216</v>
       </c>
       <c r="D68" s="2"/>
       <c r="E68" s="3" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="F68" s="2">
         <v>2</v>
       </c>
       <c r="G68" s="4">
-        <v>0.26</v>
+        <v>0.2</v>
       </c>
       <c r="H68" s="4">
-        <v>0.53</v>
+        <v>0.4</v>
       </c>
       <c r="I68" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J68" s="5" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="K68" s="3"/>
     </row>
-    <row r="69" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>248</v>
+        <v>216</v>
       </c>
       <c r="D69" s="2"/>
-      <c r="E69" s="3" t="s">
-        <v>249</v>
-      </c>
+      <c r="E69" s="3"/>
       <c r="F69" s="2">
-        <v>2</v>
-      </c>
-      <c r="G69" s="4">
-        <v>3.5</v>
-      </c>
-      <c r="H69" s="4">
-        <v>6.99</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G69" s="2"/>
+      <c r="H69" s="2"/>
       <c r="I69" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J69" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="K69" s="3"/>
-    </row>
-    <row r="70" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>213</v>
+      </c>
+      <c r="J69" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="K69" s="3" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>252</v>
+        <v>216</v>
       </c>
       <c r="D70" s="2"/>
       <c r="E70" s="3" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="F70" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G70" s="4">
-        <v>21.92</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="H70" s="4">
-        <v>21.92</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="I70" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J70" s="5" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="K70" s="3"/>
     </row>
-    <row r="71" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>256</v>
+        <v>216</v>
       </c>
       <c r="D71" s="2"/>
       <c r="E71" s="3" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="F71" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G71" s="4">
-        <v>0.21</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="H71" s="4">
-        <v>1.67</v>
+        <v>4.43</v>
       </c>
       <c r="I71" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J71" s="5" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="K71" s="3"/>
     </row>
-    <row r="72" spans="1:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>260</v>
+        <v>216</v>
       </c>
       <c r="D72" s="2"/>
       <c r="E72" s="3" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="F72" s="2">
+        <v>8</v>
+      </c>
+      <c r="G72" s="4">
+        <v>0.13</v>
+      </c>
+      <c r="H72" s="4">
+        <v>1.03</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J72" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="K72" s="3"/>
+    </row>
+    <row r="73" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D73" s="2"/>
+      <c r="E73" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="F73" s="2">
+        <v>2</v>
+      </c>
+      <c r="G73" s="4">
+        <v>0.26</v>
+      </c>
+      <c r="H73" s="4">
+        <v>0.53</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J73" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="K73" s="3"/>
+    </row>
+    <row r="74" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D74" s="2"/>
+      <c r="E74" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="F74" s="2">
+        <v>2</v>
+      </c>
+      <c r="G74" s="4">
+        <v>3.5</v>
+      </c>
+      <c r="H74" s="4">
+        <v>6.99</v>
+      </c>
+      <c r="I74" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J74" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="K74" s="3"/>
+    </row>
+    <row r="75" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="D75" s="2"/>
+      <c r="E75" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="F75" s="2">
         <v>1</v>
       </c>
-      <c r="G72" s="4">
-        <v>38.799999999999997</v>
-      </c>
-      <c r="H72" s="4">
-        <v>38.799999999999997</v>
-      </c>
-      <c r="I72" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="J72" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="K72" s="3" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A73" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="D73" s="2"/>
-      <c r="E73" s="3"/>
-      <c r="F73" s="2">
-        <v>1</v>
-      </c>
-      <c r="G73" s="2"/>
-      <c r="H73" s="2"/>
-      <c r="I73" s="2"/>
-      <c r="J73" s="3"/>
-      <c r="K73" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A74" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="D74" s="2"/>
-      <c r="E74" s="3"/>
-      <c r="F74" s="2">
-        <v>1</v>
-      </c>
-      <c r="G74" s="2"/>
-      <c r="H74" s="2"/>
-      <c r="I74" s="2"/>
-      <c r="J74" s="3"/>
-      <c r="K74" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A75" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="D75" s="2"/>
-      <c r="E75" s="3"/>
-      <c r="F75" s="2">
-        <v>2</v>
-      </c>
-      <c r="G75" s="2"/>
-      <c r="H75" s="2"/>
-      <c r="I75" s="2"/>
-      <c r="J75" s="3"/>
-      <c r="K75" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G75" s="4">
+        <v>21.92</v>
+      </c>
+      <c r="H75" s="4">
+        <v>21.92</v>
+      </c>
+      <c r="I75" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J75" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="K75" s="3"/>
+    </row>
+    <row r="76" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="D76" s="2"/>
-      <c r="E76" s="3"/>
+      <c r="E76" s="3" t="s">
+        <v>281</v>
+      </c>
       <c r="F76" s="2">
-        <v>1</v>
-      </c>
-      <c r="G76" s="2"/>
-      <c r="H76" s="2"/>
-      <c r="I76" s="2"/>
-      <c r="J76" s="3"/>
-      <c r="K76" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+      <c r="G76" s="4">
+        <v>0.21</v>
+      </c>
+      <c r="H76" s="4">
+        <v>1.67</v>
+      </c>
+      <c r="I76" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J76" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="K76" s="3"/>
+    </row>
+    <row r="77" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>270</v>
+        <v>283</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
       <c r="D77" s="2"/>
-      <c r="E77" s="3"/>
+      <c r="E77" s="3" t="s">
+        <v>285</v>
+      </c>
       <c r="F77" s="2">
         <v>1</v>
       </c>
-      <c r="G77" s="2"/>
-      <c r="H77" s="2"/>
-      <c r="I77" s="2"/>
-      <c r="J77" s="3"/>
+      <c r="G77" s="4">
+        <v>38.799999999999997</v>
+      </c>
+      <c r="H77" s="4">
+        <v>38.799999999999997</v>
+      </c>
+      <c r="I77" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="J77" s="5" t="s">
+        <v>287</v>
+      </c>
       <c r="K77" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
       <c r="D78" s="2"/>
       <c r="E78" s="3"/>
@@ -3655,18 +3810,18 @@
       <c r="I78" s="2"/>
       <c r="J78" s="3"/>
       <c r="K78" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>272</v>
+        <v>291</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
       <c r="D79" s="2"/>
       <c r="E79" s="3"/>
@@ -3678,41 +3833,41 @@
       <c r="I79" s="2"/>
       <c r="J79" s="3"/>
       <c r="K79" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>273</v>
+        <v>292</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
       <c r="D80" s="2"/>
       <c r="E80" s="3"/>
       <c r="F80" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
       <c r="I80" s="2"/>
       <c r="J80" s="3"/>
       <c r="K80" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
       <c r="D81" s="2"/>
       <c r="E81" s="3"/>
@@ -3724,18 +3879,18 @@
       <c r="I81" s="2"/>
       <c r="J81" s="3"/>
       <c r="K81" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
       <c r="D82" s="2"/>
       <c r="E82" s="3"/>
@@ -3747,20 +3902,135 @@
       <c r="I82" s="2"/>
       <c r="J82" s="3"/>
       <c r="K82" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G83" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="H83" s="7">
-        <f>SUM(H2:H82)</f>
-        <v>431.66800000000006</v>
+        <v>290</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D83" s="2"/>
+      <c r="E83" s="3"/>
+      <c r="F83" s="2">
+        <v>1</v>
+      </c>
+      <c r="G83" s="2"/>
+      <c r="H83" s="2"/>
+      <c r="I83" s="2"/>
+      <c r="J83" s="3"/>
+      <c r="K83" s="3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D84" s="2"/>
+      <c r="E84" s="3"/>
+      <c r="F84" s="2">
+        <v>1</v>
+      </c>
+      <c r="G84" s="2"/>
+      <c r="H84" s="2"/>
+      <c r="I84" s="2"/>
+      <c r="J84" s="3"/>
+      <c r="K84" s="3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A85" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D85" s="2"/>
+      <c r="E85" s="3"/>
+      <c r="F85" s="2">
+        <v>1</v>
+      </c>
+      <c r="G85" s="2"/>
+      <c r="H85" s="2"/>
+      <c r="I85" s="2"/>
+      <c r="J85" s="3"/>
+      <c r="K85" s="3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A86" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D86" s="2"/>
+      <c r="E86" s="3"/>
+      <c r="F86" s="2">
+        <v>1</v>
+      </c>
+      <c r="G86" s="2"/>
+      <c r="H86" s="2"/>
+      <c r="I86" s="2"/>
+      <c r="J86" s="3"/>
+      <c r="K86" s="3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D87" s="2"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="2">
+        <v>1</v>
+      </c>
+      <c r="G87" s="2"/>
+      <c r="H87" s="2"/>
+      <c r="I87" s="2"/>
+      <c r="J87" s="3"/>
+      <c r="K87" s="3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G88" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="H88" s="7">
+        <f>SUM(H2:H87)</f>
+        <v>438.29800000000006</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K82" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:K87" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="J2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="J3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -3810,23 +4080,23 @@
     <hyperlink ref="J49" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
     <hyperlink ref="J51" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
     <hyperlink ref="J54" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="J55" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="J56" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="J57" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="J58" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="J59" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="J60" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="J61" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="J62" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="J63" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="J65" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="J66" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="J67" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="J68" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="J69" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="J70" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="J71" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="J72" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="J56" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="J59" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="J60" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="J61" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="J62" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="J63" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="J65" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="J66" r:id="rId56" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="J67" r:id="rId57" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="J68" r:id="rId58" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="J70" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="J71" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="J72" r:id="rId61" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="J55" r:id="rId62" xr:uid="{9A9E7182-D561-448F-B3DE-713141C0DDE9}"/>
+    <hyperlink ref="J57" r:id="rId63" xr:uid="{3B839FDA-2FC5-495B-BB70-0DB6DB1ABDB8}"/>
+    <hyperlink ref="J58" r:id="rId64" xr:uid="{5CB89934-EE75-427F-8E6F-B4769E074DF0}"/>
+    <hyperlink ref="J69" r:id="rId65" xr:uid="{2C81FA5E-6AA2-4B42-9246-602C00D99655}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>